<commit_message>
WIP: Client page added
</commit_message>
<xml_diff>
--- a/Loopbaan onderzoek 5.0 template.xlsx
+++ b/Loopbaan onderzoek 5.0 template.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="120" windowWidth="15312" windowHeight="7992" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Fase 1.0 | Loopbaanfasen" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Fase 1.1 | Big Five Dimensies" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Fase 2.0 | Loopbaanankers" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Fase 2.1 | Carriere Clusters" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Fase 2.2 | Cultuur analyse" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Fase 2.3 | J.C.M." sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Rapport" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Gegevens" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fase 1.0 | Loopbaanfasen" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fase 1.1 | Big Five Dimensies" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fase 2.0 | Loopbaanankers" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fase 2.1 | Carriere Clusters" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fase 2.2 | Cultuur analyse" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fase 2.3 | J.C.M." sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rapport" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gegevens" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="152511" fullCalcOnLoad="1"/>
@@ -1151,7 +1151,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>0</col>
@@ -1169,24 +1169,24 @@
       <nvPicPr>
         <cNvPr id="2" name="Afbeelding 1"/>
         <cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </cNvPicPr>
       </nvPicPr>
       <blipFill>
-        <a:blip r:embed="rId1"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:xfrm>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:off x="0" y="1"/>
           <a:ext cx="1000125" cy="931366"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
           <avLst/>
         </a:prstGeom>
-        <a:ln>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
@@ -1197,7 +1197,7 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>2</col>
@@ -1215,24 +1215,24 @@
       <nvPicPr>
         <cNvPr id="3" name="Afbeelding 2" descr="BFP.jpg"/>
         <cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </cNvPicPr>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:xfrm>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:off x="8638760" y="10452652"/>
           <a:ext cx="6899414" cy="5441674"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
           <avLst/>
         </a:prstGeom>
-        <a:ln>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
@@ -1243,7 +1243,7 @@
 </file>
 
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>0</col>
@@ -1261,24 +1261,24 @@
       <nvPicPr>
         <cNvPr id="3" name="Afbeelding 2"/>
         <cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </cNvPicPr>
       </nvPicPr>
       <blipFill>
-        <a:blip r:embed="rId1"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:xfrm>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:off x="0" y="3878580"/>
           <a:ext cx="5848350" cy="3867150"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
           <avLst/>
         </a:prstGeom>
-        <a:ln>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
@@ -1289,7 +1289,7 @@
 </file>
 
 <file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>0</col>
@@ -1307,24 +1307,24 @@
       <nvPicPr>
         <cNvPr id="2" name="Afbeelding 1"/>
         <cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </cNvPicPr>
       </nvPicPr>
       <blipFill>
-        <a:blip r:embed="rId1"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:xfrm>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:off x="0" y="5090160"/>
           <a:ext cx="6461760" cy="4861560"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
           <avLst/>
         </a:prstGeom>
-        <a:ln>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
@@ -2246,7 +2246,7 @@
       </c>
       <c r="C5" s="28" t="n"/>
       <c r="D5" s="29" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E5" s="28" t="n"/>
       <c r="F5" s="28" t="n"/>
@@ -2264,7 +2264,7 @@
       <c r="C6" s="28" t="n"/>
       <c r="D6" s="28" t="n"/>
       <c r="E6" s="30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F6" s="28" t="n"/>
       <c r="G6" s="32" t="n"/>
@@ -2282,7 +2282,7 @@
       <c r="D7" s="28" t="n"/>
       <c r="E7" s="28" t="n"/>
       <c r="F7" s="31" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G7" s="32" t="n"/>
     </row>
@@ -2300,7 +2300,7 @@
       <c r="E8" s="28" t="n"/>
       <c r="F8" s="28" t="n"/>
       <c r="G8" s="33" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -2313,7 +2313,7 @@
         </is>
       </c>
       <c r="C9" s="27" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D9" s="28" t="n"/>
       <c r="E9" s="28" t="n"/>
@@ -2331,7 +2331,7 @@
       </c>
       <c r="C10" s="28" t="n"/>
       <c r="D10" s="29" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E10" s="28" t="n"/>
       <c r="F10" s="28" t="n"/>
@@ -2349,7 +2349,7 @@
       <c r="C11" s="28" t="n"/>
       <c r="D11" s="28" t="n"/>
       <c r="E11" s="30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F11" s="28" t="n"/>
       <c r="G11" s="32" t="n"/>
@@ -2367,7 +2367,7 @@
       <c r="D12" s="28" t="n"/>
       <c r="E12" s="28" t="n"/>
       <c r="F12" s="31" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G12" s="32" t="n"/>
     </row>
@@ -2385,7 +2385,7 @@
       <c r="E13" s="28" t="n"/>
       <c r="F13" s="28" t="n"/>
       <c r="G13" s="33" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -2398,7 +2398,7 @@
         </is>
       </c>
       <c r="C14" s="27" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D14" s="28" t="n"/>
       <c r="E14" s="28" t="n"/>
@@ -2416,7 +2416,7 @@
       </c>
       <c r="C15" s="28" t="n"/>
       <c r="D15" s="29" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E15" s="28" t="n"/>
       <c r="F15" s="28" t="n"/>
@@ -2434,7 +2434,7 @@
       <c r="C16" s="28" t="n"/>
       <c r="D16" s="28" t="n"/>
       <c r="E16" s="30" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F16" s="28" t="n"/>
       <c r="G16" s="32" t="n"/>
@@ -2452,7 +2452,7 @@
       <c r="D17" s="28" t="n"/>
       <c r="E17" s="28" t="n"/>
       <c r="F17" s="31" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G17" s="32" t="n"/>
     </row>
@@ -2470,7 +2470,7 @@
       <c r="E18" s="28" t="n"/>
       <c r="F18" s="28" t="n"/>
       <c r="G18" s="33" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19">
@@ -2483,7 +2483,7 @@
         </is>
       </c>
       <c r="C19" s="27" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D19" s="28" t="n"/>
       <c r="E19" s="28" t="n"/>
@@ -2501,7 +2501,7 @@
       </c>
       <c r="C20" s="28" t="n"/>
       <c r="D20" s="29" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E20" s="28" t="n"/>
       <c r="F20" s="28" t="n"/>
@@ -2519,7 +2519,7 @@
       <c r="C21" s="28" t="n"/>
       <c r="D21" s="28" t="n"/>
       <c r="E21" s="30" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F21" s="28" t="n"/>
       <c r="G21" s="32" t="n"/>
@@ -2537,7 +2537,7 @@
       <c r="D22" s="28" t="n"/>
       <c r="E22" s="28" t="n"/>
       <c r="F22" s="31" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G22" s="32" t="n"/>
     </row>
@@ -2555,7 +2555,7 @@
       <c r="E23" s="28" t="n"/>
       <c r="F23" s="28" t="n"/>
       <c r="G23" s="33" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="24">
@@ -2568,7 +2568,7 @@
         </is>
       </c>
       <c r="C24" s="27" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D24" s="28" t="n"/>
       <c r="E24" s="28" t="n"/>
@@ -2586,7 +2586,7 @@
       </c>
       <c r="C25" s="28" t="n"/>
       <c r="D25" s="29" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E25" s="28" t="n"/>
       <c r="F25" s="28" t="n"/>
@@ -2604,7 +2604,7 @@
       <c r="C26" s="28" t="n"/>
       <c r="D26" s="28" t="n"/>
       <c r="E26" s="30" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F26" s="28" t="n"/>
       <c r="G26" s="32" t="n"/>
@@ -2792,7 +2792,7 @@
       <c r="D37" s="28" t="n"/>
       <c r="E37" s="28" t="n"/>
       <c r="F37" s="31" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G37" s="32" t="n"/>
     </row>
@@ -2810,7 +2810,7 @@
       <c r="E38" s="28" t="n"/>
       <c r="F38" s="28" t="n"/>
       <c r="G38" s="33" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="39">
@@ -2823,7 +2823,7 @@
         </is>
       </c>
       <c r="C39" s="27" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D39" s="28" t="n"/>
       <c r="E39" s="28" t="n"/>
@@ -2841,7 +2841,7 @@
       </c>
       <c r="C40" s="28" t="n"/>
       <c r="D40" s="29" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E40" s="28" t="n"/>
       <c r="F40" s="28" t="n"/>
@@ -2859,7 +2859,7 @@
       <c r="C41" s="28" t="n"/>
       <c r="D41" s="28" t="n"/>
       <c r="E41" s="30" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F41" s="28" t="n"/>
       <c r="G41" s="32" t="n"/>
@@ -2877,7 +2877,7 @@
       <c r="D42" s="28" t="n"/>
       <c r="E42" s="28" t="n"/>
       <c r="F42" s="31" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G42" s="32" t="n"/>
     </row>
@@ -2895,7 +2895,7 @@
       <c r="E43" s="28" t="n"/>
       <c r="F43" s="28" t="n"/>
       <c r="G43" s="33" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="44">
@@ -2908,7 +2908,7 @@
         </is>
       </c>
       <c r="C44" s="27" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D44" s="28" t="n"/>
       <c r="E44" s="28" t="n"/>
@@ -2926,7 +2926,7 @@
       </c>
       <c r="C45" s="28" t="n"/>
       <c r="D45" s="29" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E45" s="28" t="n"/>
       <c r="F45" s="28" t="n"/>
@@ -2944,7 +2944,7 @@
       <c r="C46" s="28" t="n"/>
       <c r="D46" s="28" t="n"/>
       <c r="E46" s="30" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F46" s="28" t="n"/>
       <c r="G46" s="32" t="n"/>
@@ -2962,7 +2962,7 @@
       <c r="D47" s="28" t="n"/>
       <c r="E47" s="28" t="n"/>
       <c r="F47" s="31" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G47" s="32" t="n"/>
     </row>
@@ -2980,7 +2980,7 @@
       <c r="E48" s="28" t="n"/>
       <c r="F48" s="28" t="n"/>
       <c r="G48" s="33" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="49">
@@ -2993,7 +2993,7 @@
         </is>
       </c>
       <c r="C49" s="27" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D49" s="28" t="n"/>
       <c r="E49" s="28" t="n"/>
@@ -3011,7 +3011,7 @@
       </c>
       <c r="C50" s="28" t="n"/>
       <c r="D50" s="29" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E50" s="28" t="n"/>
       <c r="F50" s="28" t="n"/>
@@ -3029,7 +3029,7 @@
       <c r="C51" s="28" t="n"/>
       <c r="D51" s="28" t="n"/>
       <c r="E51" s="30" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F51" s="28" t="n"/>
       <c r="G51" s="32" t="n"/>
@@ -3047,7 +3047,7 @@
       <c r="D52" s="28" t="n"/>
       <c r="E52" s="28" t="n"/>
       <c r="F52" s="31" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G52" s="32" t="n"/>
     </row>
@@ -3065,7 +3065,7 @@
       <c r="E53" s="28" t="n"/>
       <c r="F53" s="28" t="n"/>
       <c r="G53" s="33" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="54">
@@ -5031,9 +5031,9 @@
   </sheetData>
   <mergeCells count="221">
     <mergeCell ref="C30:C31"/>
+    <mergeCell ref="D53:D55"/>
     <mergeCell ref="E39:E40"/>
     <mergeCell ref="D60:D63"/>
-    <mergeCell ref="D53:D55"/>
     <mergeCell ref="F60:F63"/>
     <mergeCell ref="E48:E49"/>
     <mergeCell ref="G48:G49"/>

</xml_diff>